<commit_message>
EOD chain Sat 7/18 catch-up run: FAST variant on Friday settled closes - zero new fresh buys; carried plan set stands
Weekend catch-up of the missed Friday run. Chart-scanned 32 fresh-tab
origination names (Buy Zone 8, Fresh Ignitions 4, Coiled convergence-
filtered to biotech/healthcare 20); reused the Friday 250-name watchlist
sweep + smoke-test reads (identical settled data, disclosed in notes).
Results JSON + xlsx regenerated; 6 wired alerts stand, no new plans.
Blockers logged in JSON: NUVL unresolvable (delisted?), 5-min feed drop
(recovered), HA-close price caveat.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/universe_2026-07-18.xlsx
+++ b/reports/universe_2026-07-18.xlsx
@@ -426,23 +426,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
     <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="58" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
     <col width="60" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
@@ -526,52 +526,442 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>NUE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>~2026-07-14</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>234.35</v>
+      </c>
+      <c r="E2" t="n">
+        <v>230.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>217.5</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>HALF $45k</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>247 -&gt; 258</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Q2 7/27 AMC pre-guided -&gt; trim 7/24</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>FULL PASS (+27.3% vs 200d, ADX 20.4, RS +36.1)</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>ACTIVE - priority #1</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Only full regime pass of the set; HRC price hike + KeyBanc upgrade; V-bottom holding. Entry 1.6% below Fri close.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>XPO</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>~2026-07-13</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>216.5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>208</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="G3" t="n">
+        <v>195.9</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>HALF $43k</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>2500</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>232</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Q2 7/30 BMO -&gt; trim 7/29</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>202</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>PASS w/ ADX 11.6 trendless flag</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>ACTIVE - priority #2</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>NO CHASE - Magical +202 very hot; pullback limit only. LTL tonnage improving; crowded-expectations print risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>950.12</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>928-930</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>902</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>STARTER $50k (downgraded from $100k)</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>2500</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>970 -&gt; 1005</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>~late Sept (clear)</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>MARGINAL FAIL - borderline vs 200d (reclaim attempt Fri)</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>ACTIVE - starter</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Fired Friday, strongest signal of the scan; full size only on a daily close above ~957 (the 200d). Bernstein top-pick catalyst.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AMT</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>~2026-07-13</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>170.9</v>
+      </c>
+      <c r="E5" t="n">
+        <v>168.5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>163.2</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>STARTER $30k (downgraded)</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>950</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>180+ (Wolfe 188 / GS 215)</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Q2 7/28 BMO -&gt; trim 7/27</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>FAIL - repair trade (-5.5% vs 200d, ADX 34)</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>ACTIVE - starter</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Upgrade cluster keeps it alive; low-vol stair-stepper; re-add post-print.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>~2026-07-14</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>249.75</v>
+      </c>
+      <c r="E6" t="n">
+        <v>245</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="G6" t="n">
+        <v>227</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>WATCH / spec-starter $25k max</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>1800</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>266 -&gt; 285</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Q2 8/6 BMO -&gt; trim 8/5</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>-42.3</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>DEEP FAIL (-19.3% vs 200d) - repair-stage chart</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>PJM auction at cap = real capacity-revenue catalyst but the base needs work; alert stands as lookpoint. Chosen vehicle over TLN (concentration rule).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>25.27</v>
+      </c>
+      <c r="E7" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="G7" t="n">
+        <v>23.55</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>~27</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Q2 8/4 BMO + PDUFA 8/17 BINARY</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>149.2</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>FAIL (-3.2% vs 200d) + binaries + hot Magical</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Weakest case of the set; alert = lookpoint only; Omar decides any PDUFA hold-through.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>FNB</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Fresh Ignitions</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>~2026-07-15 (2-3 sessions old)</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>~2026-07-15</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
         <v>18.99</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G8" t="n">
         <v>18.51</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H8" t="n">
         <v>0</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I8" t="n">
         <v>0</v>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>REPORTED Q2 2026-07-16 AMC - beat (EPS $0.42 +17% y/y, record revenue $462.7M) but shares slipped on the print; no upcoming binary</t>
-        </is>
-      </c>
-      <c r="L2" t="n">
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>REPORTED Q2 2026-07-16 AMC - beat (EPS $0.42, record revenue) but faded on the print; no upcoming binary</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
         <v>19.3</v>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>not run (test mode - light gates)</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>not run - ZLSMA gate already fails</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
         <is>
           <t>watch</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>ZLSMA gate FAIL: last 18.99 &lt; ZLSMA(50) 19.71. Friday was a high-volume post-earnings fade (-1.6% on 19M shares vs ~7M avg) despite the beat. CE long stop 18.51 held (Fri low 18.80). No plan, no alert - reassess if price reclaims ZLSMA ~19.7.</t>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>ZLSMA gate FAIL (18.99 &lt; 19.71); Friday high-volume post-earnings fade despite the beat; CE long stop 18.51 held. Reassess on reclaim of ~19.7. Still in the fresh 7/18 Fresh Ignitions tab.</t>
         </is>
       </c>
     </row>
@@ -586,13 +976,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -614,6 +1004,270 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>HAS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>~2026-07-14</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Earnings Tue 7/21 BMO = rule 6 (no entry day-before a print); PT-cut cluster into it. Re-check the O.G read after the print.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>~2026-07-13</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ZLSMA FAIL as of Fri close (1,067 &lt; 1,080) + Friday retraced nearly the whole record-earnings gap. Watch: reclaim 1,080 + hold 1,047.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CVNA</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>~2026-07-15</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ZLSMA FAIL (68.4 &lt; 70.8) + earnings 7/29 within 7 sessions + priced-for-perfection. Re-look post-print.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BHP</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>~2026-07-13</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Signal real but catalyst NEGATIVE (FY27 copper guide cut drove the fade into the signal). Watch-only: needs a green day holding 78.66.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TLN</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>~2026-07-14</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Friday low pierced the signal level intraday; 6.5% ATR; same PJM theme as CEG with a worse chart - CEG is the vehicle (concentration rule).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LCID</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Solvency-headline binary (bankruptcy report 7/14, denied) + Magical +135 hot. Spec bucket at best - SKIP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SHAK</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>~2026-07-13</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Deep ZLSMA FAIL (58.5 vs 72.5) + June guidance cut = show-me story. Watch the base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SPXL</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>~2026-07-10 (borderline, 5 bars)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>3x-levered index vehicle, weakest freshness of the set, Friday -3.3% back near signal - not a plan candidate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SION</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Fresh Ignitions</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>no (signal ~2026-06-23)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Long mode but stale signal + Magical +160 chasing-hot. No fresh entry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ESQ</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Fresh Ignitions</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>no (signal ~2026-05-20)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Long mode, stale signal, Magical +158 chasing-hot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DX</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Fresh Ignitions</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>no (signal ~2026-06-18)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Long mode, stale signal, Magical +174 chasing-hot; mortgage REIT (yield vehicle, not a swing chart).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>COCO</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>no (~2026-07-09, 6 sessions)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Near-miss: buy one session outside the 5-bar window; long stop 64.72 vs last 73.01. On deck if it holds.</t>
         </is>
       </c>
     </row>
@@ -628,7 +1282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -644,96 +1298,1062 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>ACGL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EXTR</t>
+          <t>AMD</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>VISN</t>
+          <t>APH</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>BWXT</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NWPX</t>
+          <t>CAT</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AMBQ</t>
+          <t>CDNS</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MEC</t>
+          <t>CHTR</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>COKE</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RAL</t>
+          <t>CPRT</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GTX</t>
+          <t>DE</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>WRLD</t>
+          <t>DELL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>DHI</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>EME</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
+        <is>
+          <t>ERIE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>FTAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>GE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>IBKR</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>LDOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>LEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MLI</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>MTZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>PGR</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>PH</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>POWL</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>RMD</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SFM</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>SHW</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>STRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>TDY</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>TPR</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>TT</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>URI</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>VRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>WMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ZTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BOTZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>CCJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>CCL</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>CRCL</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>GEV</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>HUBB</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>JETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>LHX</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>LUNR</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>LUV</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>NCLH</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>OKLO</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>PWR</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>RCL</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ROBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>SMR</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>UAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>URA</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ALB</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>AROC</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>BBAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>BCBP</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>BROS</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>BTBT</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>BTCS</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>CBRS</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>CENX</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>CLX</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>CRWV</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>CSCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>CTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>DGX</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>DTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>EVGO</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>FCX</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>FHB</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>FLEX</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>FSLR</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>FUTU</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>HIMX</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>HTZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>HUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>HYPD</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>INOD</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>LAES</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>MCHP</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>NEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>NIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>NVAX</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>NVTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>OILD</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>ORBS</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>PURR</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>RGTI</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>SMH</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>SMMT</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>SOUN</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>UAVS</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>VMI</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>XLK</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>OSCR</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>MIRM</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>BIOA</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>SRRK</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>KURA</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>PTCT</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>IRMD</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>MLAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>EXTR</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>VISN</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>NWPX</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>GTX</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
         <is>
           <t>NVST</t>
         </is>
@@ -789,7 +2409,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>fast</t>
         </is>
       </c>
     </row>
@@ -800,7 +2420,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26</v>
+        <v>289</v>
       </c>
     </row>
     <row r="5">
@@ -810,7 +2430,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -820,7 +2440,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -830,7 +2450,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -840,7 +2460,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>14</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9">
@@ -850,7 +2470,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>8900</v>
       </c>
     </row>
     <row r="10">
@@ -861,7 +2481,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SMOKE TEST of the autonomous chain (Omar-directed): origination Buy Zone (19) + Fresh Ignitions (7) tabs only; Coiled and the three watchlists deliberately skipped. Origination tabs exported 2026-07-18 but xlsx basis is 2026-07-16 15:50 (Wed close) - tab membership is 2 sessions stale. Market closed (Sat); latest bar = Fri 2026-07-17 as expected. Chain health: TV feed up, layout_switch to O.G Chandelier id 91698392 verified via chart_get_state (Volume/ZLSMA/Chandelier/Magical), all 26 symbols resolved to correct US listings (LTC = LTC Properties NYSE, not Litecoin; GGB = Gerdau NYSE ADR), no blockers, no user input needed. Broad-tape read: 14 of 26 names in CE sell mode with deep negative Magical readings (AMD -190, AMBQ -247, MEC -220, DELL -148) - Thu/Fri pullback washed out most of the Buy Zone tab. Near-miss: COCO buy ~2026-07-09 (~6 sessions, just outside the 5-session window), long stop 64.72, last 73.01, still long mode. Gates run LIGHT per test directive: earnings via one web check on the single hit; HQ Swing regime scanner call NOT run. BLOCKER (logged per autonomous-run rule): git commit DENIED by session permission mode (dont-ask) - git status/add worked, commit refused on 3 attempts; JSON + reports/universe_2026-07-18.xlsx left STAGED on branch add-watchlist-files for Omar to commit. Also note: compile_daily_report.py ran fine via Bash but PowerShell tool was denied - the real EOD chain runs it from the bat, so no chain impact.</t>
+          <t>SATURDAY CATCH-UP RUN of the missed Friday EOD chain (weekend rule: fast convergence variant on latest settled data = Friday 2026-07-17 closes; no new bars have printed since). Universe 289 = three watchlists (250) + fresh 2026-07-18 origination tabs (Buy Zone 16 / Fresh Ignitions 6 / Coiled convergence-filtered to radar WATCH-or-IGNITING sectors = 24 biotech/healthcare names; radar 7/17: XBI/IBB/XLV WATCH + KWEB IGNITING, but Coiled holds zero China-internet names). CHART WORK THIS RUN: 32 origination names not previously read on this data, scanned live on the O.G Chandelier layout (id 91698392, stack verified) -&gt; ZERO new fresh buys (14 long-but-stale + 2 sell in Buy-Zone/FI chunk; 7 long-but-stale + 8 sell in Coiled-biotech chunk). REUSED ON IDENTICAL SETTLED DATA (disclosed per catch-up rule): the 250-name watchlist sweep from og-chandelier-scan-2026-07-17.md (run Friday post-close on these same closes) and today's earlier smoke-test reads (FNB hit-&gt;watch; NWPX/EXTR/VISN/GTX/NVST sell; COCO long ~7/9 just outside window). Hits below = the carried 7/17 signal set with plans from research/plans-2026-07-20.md including the Sat regime retro-check downgrades (NUE priority 1 full-pass; COST/AMT starters; CEG/PFE watch); the 6 entry alerts already wired Fri stand - NO new alerts wired this run (nothing new to wire). Combined risk if all actives fill ~$8.9k, under the $10k weekly flag. BLOCKERS/CAVEATS LOGGED (autonomous rule, no user input): (1) NUVL (Coiled) unresolvable on NASDAQ/NYSE - possibly delisted/acquired, needs Omar to confirm and clean the scanner universe; (2) TV feed dropped ~5 min mid-scan and again briefly during quote pulls - self-recovered, chunk restarted, no data gaps; (3) O.G layout is a Heikin-Ashi chart, so 'last' prices are HA composite closes off Omar's own layout (COST/PFE cross-check plan prices exactly; treat sub-1% entry distances as approximate); (4) quote_get returns stale prior-symbol data after symbol switches when market closed - worked around via data_get_ohlcv with readiness retries; (5) pine/~$ctor_rotation_detector.pine (Office temp lock file) left uncommitted deliberately. Buy-Zone tab character note for the tracker: all 8 newly-scanned Buy-Zone names are in LONG mode from mid-May/June signals now pulling back (that is what the tab screens for) - the O.G fresh-buy overlay found nothing &lt;=5 sessions old among them; SION/ESQ/DX (Fresh Ignitions) long but Magical +158/+158/+174 = chasing-hot, no entry.</t>
         </is>
       </c>
     </row>

</xml_diff>